<commit_message>
exp max new tokens modified results
</commit_message>
<xml_diff>
--- a/results/reliability_eval/reliability_eval_09-17-1-test/Llama-3-8B_P101_0_sample_25_tokens_0.1_temp_original_raw_table_09-17-1-test.xlsx
+++ b/results/reliability_eval/reliability_eval_09-17-1-test/Llama-3-8B_P101_0_sample_25_tokens_0.1_temp_original_raw_table_09-17-1-test.xlsx
@@ -650,31 +650,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>A. He is an expert in the field of physics. B. He is an expert in the field of mathematics. C</t>
+          <t>What is John Vincent Atanasoff's area of expertise?
+John Vincent Atanasoff's area of expertise is in the field</t>
         </is>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2270916998386383</v>
+        <v>0.3486451208591461</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9424276947975159</v>
+        <v>0.9587278366088867</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6466038227081299</v>
+        <v>0.3673676252365112</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>[(' A', 0.6514), ('.', 1.0), (' He', 0.3486), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' in', 1.0), (' the', 1.0), (' field', 1.0), (' of', 1.0), (' physics', 1.0), ('.', 1.0), (' B', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' in', 1.0), (' the', 1.0), (' field', 1.0), (' of', 1.0), (' mathematics', 1.0), ('.', 1.0), (' C', 1.0)]</t>
+          <t>[(' What', 0.3486), (' is', 1.0), (' John', 1.0), (' Vincent', 1.0), (' At', 1.0), ('anas', 1.0), ('off', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?\n', 1.0), ('John', 1.0), (' Vincent', 1.0), (' At', 1.0), ('anas', 1.0), ('off', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), (' is', 1.0), (' in', 1.0), (' the', 1.0), (' field', 1.0)]</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -696,78 +697,78 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>A. John Vincent Atanasoff's area of expertise is in the field of physics. B. John Vincent Atanasoff</t>
+        </is>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.424263209104538</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.9662854075431824</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.5584724545478821</v>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>[(' A', 0.6514), ('.', 1.0), (' John', 0.6514), (' Vincent', 1.0), (' At', 1.0), ('anas', 1.0), ('off', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), (' is', 1.0), (' in', 1.0), (' the', 1.0), (' field', 1.0), (' of', 1.0), (' physics', 1.0), ('.', 1.0), (' B', 1.0), ('.', 1.0), (' John', 1.0), (' Vincent', 1.0), (' At', 1.0), ('anas', 1.0), ('off', 1.0)]</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>What is John Vincent Atanasoff's area of expertise?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>mathematics</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>What is John Vincent Atanasoff's area of expertise?
 John Vincent Atanasoff's area of expertise is in the field</t>
         </is>
       </c>
-      <c r="F6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" t="n">
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
         <v>0.3486451208591461</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H7" t="n">
         <v>0.9587278366088867</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I7" t="n">
         <v>0.3673676252365112</v>
       </c>
-      <c r="J6" t="b">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr">
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>[(' What', 0.3486), (' is', 1.0), (' John', 1.0), (' Vincent', 1.0), (' At', 1.0), ('anas', 1.0), ('off', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?\n', 1.0), ('John', 1.0), (' Vincent', 1.0), (' At', 1.0), ('anas', 1.0), ('off', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), (' is', 1.0), (' in', 1.0), (' the', 1.0), (' field', 1.0)]</t>
         </is>
       </c>
-      <c r="L6" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>What is John Vincent Atanasoff's area of expertise?</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>mathematics</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>A. John Vincent Atanasoff's area of expertise is in the field of physics. B. John Vincent Atanasoff</t>
-        </is>
-      </c>
-      <c r="F7" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.424263209104538</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.9662854075431824</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.5584724545478821</v>
-      </c>
-      <c r="J7" t="b">
-        <v>0</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>[(' A', 0.6514), ('.', 1.0), (' John', 0.6514), (' Vincent', 1.0), (' At', 1.0), ('anas', 1.0), ('off', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), (' is', 1.0), (' in', 1.0), (' the', 1.0), (' field', 1.0), (' of', 1.0), (' physics', 1.0), ('.', 1.0), (' B', 1.0), ('.', 1.0), (' John', 1.0), (' Vincent', 1.0), (' At', 1.0), ('anas', 1.0), ('off', 1.0)]</t>
-        </is>
-      </c>
       <c r="L7" t="n">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -789,8 +790,8 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>A. Anthropology B. Archaeology C. Sociology D. Psychology
-What is Edward Burnett Tylor's area of</t>
+          <t>A. anthropology B. archaeology C. paleontology D. geology
+What is Edward Burnett Tylor's area</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -810,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>[(' A', 1.0), ('.', 1.0), (' Anthrop', 0.5), ('ology', 1.0), (' B', 1.0), ('.', 1.0), (' Archae', 1.0), ('ology', 1.0), (' C', 1.0), ('.', 1.0), (' Sociology', 1.0), (' D', 1.0), ('.', 1.0), (' Psychology', 1.0), ('\n', 1.0), ('What', 1.0), (' is', 1.0), (' Edward', 1.0), (' Burnett', 1.0), (' T', 1.0), ('yl', 1.0), ('or', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0)]</t>
+          <t>[(' A', 1.0), ('.', 1.0), (' anthropology', 0.5), (' B', 1.0), ('.', 1.0), (' archae', 1.0), ('ology', 1.0), (' C', 1.0), ('.', 1.0), (' pale', 1.0), ('ontology', 1.0), (' D', 1.0), ('.', 1.0), (' ge', 1.0), ('ology', 1.0), ('\n', 1.0), ('What', 1.0), (' is', 1.0), (' Edward', 1.0), (' Burnett', 1.0), (' T', 1.0), ('yl', 1.0), ('or', 1.0), ("'s", 1.0), (' area', 1.0)]</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -931,27 +932,27 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>What is his area of expertise?
-Anaxagoras is a philosopher who lived in the 5th century BC. He</t>
+Anaxagoras is a Greek philosopher who lived in the 5th century BC.</t>
         </is>
       </c>
       <c r="F11" t="b">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3486451208591461</v>
+        <v>0.6513549089431763</v>
       </c>
       <c r="H11" t="n">
-        <v>0.9587278366088867</v>
+        <v>0.9829981923103333</v>
       </c>
       <c r="I11" t="n">
-        <v>0.3673676252365112</v>
+        <v>0.279236227273941</v>
       </c>
       <c r="J11" t="b">
         <v>0</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>[(' What', 1.0), (' is', 1.0), (' his', 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?\n', 1.0), ('An', 1.0), ('ax', 1.0), ('ag', 1.0), ('oras', 1.0), (' is', 1.0), (' a', 1.0), (' philosopher', 0.3486), (' who', 1.0), (' lived', 1.0), (' in', 1.0), (' the', 1.0), (' ', 1.0), ('5', 1.0), ('th', 1.0), (' century', 1.0), (' BC', 1.0), ('.', 1.0), (' He', 1.0)]</t>
+          <t>[(' What', 1.0), (' is', 1.0), (' his', 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?\n', 1.0), ('An', 1.0), ('ax', 1.0), ('ag', 1.0), ('oras', 1.0), (' is', 1.0), (' a', 1.0), (' Greek', 0.6514), (' philosopher', 1.0), (' who', 1.0), (' lived', 1.0), (' in', 1.0), (' the', 1.0), (' ', 1.0), ('5', 1.0), ('th', 1.0), (' century', 1.0), (' BC', 1.0), ('.', 1.0)]</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -978,27 +979,27 @@
       <c r="E12" t="inlineStr">
         <is>
           <t>What is his area of expertise?
-Anaxagoras is a philosopher who lived in the 5th century BC. He</t>
+Anaxagoras is a Greek philosopher who lived in the 5th century BC.</t>
         </is>
       </c>
       <c r="F12" t="b">
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3486451208591461</v>
+        <v>0.6513549089431763</v>
       </c>
       <c r="H12" t="n">
-        <v>0.9587278366088867</v>
+        <v>0.9829981923103333</v>
       </c>
       <c r="I12" t="n">
-        <v>0.3673676252365112</v>
+        <v>0.279236227273941</v>
       </c>
       <c r="J12" t="b">
         <v>0</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>[(' What', 1.0), (' is', 1.0), (' his', 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?\n', 1.0), ('An', 1.0), ('ax', 1.0), ('ag', 1.0), ('oras', 1.0), (' is', 1.0), (' a', 1.0), (' philosopher', 0.3486), (' who', 1.0), (' lived', 1.0), (' in', 1.0), (' the', 1.0), (' ', 1.0), ('5', 1.0), ('th', 1.0), (' century', 1.0), (' BC', 1.0), ('.', 1.0), (' He', 1.0)]</t>
+          <t>[(' What', 1.0), (' is', 1.0), (' his', 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?\n', 1.0), ('An', 1.0), ('ax', 1.0), ('ag', 1.0), ('oras', 1.0), (' is', 1.0), (' a', 1.0), (' Greek', 0.6514), (' philosopher', 1.0), (' who', 1.0), (' lived', 1.0), (' in', 1.0), (' the', 1.0), (' ', 1.0), ('5', 1.0), ('th', 1.0), (' century', 1.0), (' BC', 1.0), ('.', 1.0)]</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1025,27 +1026,27 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>What is his area of expertise?
-Anaxagoras is a philosopher who lived in the 5th century BC. He</t>
+Anaxagoras is a Greek philosopher who lived in the 5th century BC.</t>
         </is>
       </c>
       <c r="F13" t="b">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0.3486451208591461</v>
+        <v>0.6513549089431763</v>
       </c>
       <c r="H13" t="n">
-        <v>0.9587278366088867</v>
+        <v>0.9829981923103333</v>
       </c>
       <c r="I13" t="n">
-        <v>0.3673676252365112</v>
+        <v>0.279236227273941</v>
       </c>
       <c r="J13" t="b">
         <v>0</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>[(' What', 1.0), (' is', 1.0), (' his', 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?\n', 1.0), ('An', 1.0), ('ax', 1.0), ('ag', 1.0), ('oras', 1.0), (' is', 1.0), (' a', 1.0), (' philosopher', 0.3486), (' who', 1.0), (' lived', 1.0), (' in', 1.0), (' the', 1.0), (' ', 1.0), ('5', 1.0), ('th', 1.0), (' century', 1.0), (' BC', 1.0), ('.', 1.0), (' He', 1.0)]</t>
+          <t>[(' What', 1.0), (' is', 1.0), (' his', 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?\n', 1.0), ('An', 1.0), ('ax', 1.0), ('ag', 1.0), ('oras', 1.0), (' is', 1.0), (' a', 1.0), (' Greek', 0.6514), (' philosopher', 1.0), (' who', 1.0), (' lived', 1.0), (' in', 1.0), (' the', 1.0), (' ', 1.0), ('5', 1.0), ('th', 1.0), (' century', 1.0), (' BC', 1.0), ('.', 1.0)]</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1212,29 +1213,27 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>What is Adam Carolla's area of expertise?
-What is Adam Carolla's area of expertise?
-Adam Carolla is a</t>
+          <t>What is his area of expertise? What is Adam Carolla's area of expertise? What is Adam Carolla's area of</t>
         </is>
       </c>
       <c r="F17" t="b">
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>0.2270916998386383</v>
+        <v>0.3486451208591461</v>
       </c>
       <c r="H17" t="n">
-        <v>0.9424276947975159</v>
+        <v>0.9587278366088867</v>
       </c>
       <c r="I17" t="n">
-        <v>0.6466038227081299</v>
+        <v>0.3673676252365112</v>
       </c>
       <c r="J17" t="b">
         <v>0</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>[(' What', 1.0), (' is', 1.0), (' Adam', 0.6514), (' Car', 1.0), ('olla', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?\n', 1.0), ('What', 1.0), (' is', 1.0), (' Adam', 1.0), (' Car', 1.0), ('olla', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?\n', 1.0), ('Adam', 0.3486), (' Car', 1.0), ('olla', 1.0), (' is', 1.0), (' a', 1.0)]</t>
+          <t>[(' What', 1.0), (' is', 1.0), (' his', 0.3486), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?', 1.0), (' What', 1.0), (' is', 1.0), (' Adam', 1.0), (' Car', 1.0), ('olla', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0), (' expertise', 1.0), ('?', 1.0), (' What', 1.0), (' is', 1.0), (' Adam', 1.0), (' Car', 1.0), ('olla', 1.0), ("'s", 1.0), (' area', 1.0), (' of', 1.0)]</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1354,27 +1353,27 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>A. He is an expert on the history of the United States. B. He is an expert on the history of the</t>
+          <t>A. He is an expert in the field of cartooning. B. He is an expert in the field of cartooning</t>
         </is>
       </c>
       <c r="F20" t="b">
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="H20" t="n">
-        <v>0.9460576772689819</v>
+        <v>0.9726549386978149</v>
       </c>
       <c r="I20" t="n">
-        <v>0.6931471824645996</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J20" t="b">
         <v>0</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>[(' A', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' on', 0.5), (' the', 1.0), (' history', 1.0), (' of', 1.0), (' the', 1.0), (' United', 0.5), (' States', 1.0), ('.', 1.0), (' B', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' on', 1.0), (' the', 1.0), (' history', 1.0), (' of', 1.0), (' the', 1.0)]</t>
+          <t>[(' A', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' in', 0.5), (' the', 1.0), (' field', 1.0), (' of', 1.0), (' cartoon', 1.0), ('ing', 1.0), ('.', 1.0), (' B', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' in', 1.0), (' the', 1.0), (' field', 1.0), (' of', 1.0), (' cartoon', 1.0), ('ing', 1.0)]</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -1400,27 +1399,27 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>A. He is an expert on the history of the American comic strip. B. He is an expert on the history of</t>
+          <t>A. He is an expert in the field of cartooning. B. He is an expert in the field of cartooning</t>
         </is>
       </c>
       <c r="F21" t="b">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="H21" t="n">
-        <v>0.9460576772689819</v>
+        <v>0.9726549386978149</v>
       </c>
       <c r="I21" t="n">
-        <v>0.6931471824645996</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J21" t="b">
         <v>0</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>[(' A', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' on', 0.5), (' the', 1.0), (' history', 1.0), (' of', 1.0), (' the', 1.0), (' American', 0.5), (' comic', 1.0), (' strip', 1.0), ('.', 1.0), (' B', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' on', 1.0), (' the', 1.0), (' history', 1.0), (' of', 1.0)]</t>
+          <t>[(' A', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' in', 0.5), (' the', 1.0), (' field', 1.0), (' of', 1.0), (' cartoon', 1.0), ('ing', 1.0), ('.', 1.0), (' B', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' in', 1.0), (' the', 1.0), (' field', 1.0), (' of', 1.0), (' cartoon', 1.0), ('ing', 1.0)]</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -1446,27 +1445,27 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>A. He is an expert on the history of the American comic strip. B. He is an expert on the history of</t>
+          <t>A. He is an expert in the field of cartooning. B. He is an expert in the field of cartooning</t>
         </is>
       </c>
       <c r="F22" t="b">
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="H22" t="n">
-        <v>0.9460576772689819</v>
+        <v>0.9726549386978149</v>
       </c>
       <c r="I22" t="n">
-        <v>0.6931471824645996</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J22" t="b">
         <v>0</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>[(' A', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' on', 0.5), (' the', 1.0), (' history', 1.0), (' of', 1.0), (' the', 1.0), (' American', 0.5), (' comic', 1.0), (' strip', 1.0), ('.', 1.0), (' B', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' on', 1.0), (' the', 1.0), (' history', 1.0), (' of', 1.0)]</t>
+          <t>[(' A', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' in', 0.5), (' the', 1.0), (' field', 1.0), (' of', 1.0), (' cartoon', 1.0), ('ing', 1.0), ('.', 1.0), (' B', 1.0), ('.', 1.0), (' He', 1.0), (' is', 1.0), (' an', 1.0), (' expert', 1.0), (' in', 1.0), (' the', 1.0), (' field', 1.0), (' of', 1.0), (' cartoon', 1.0), ('ing', 1.0)]</t>
         </is>
       </c>
       <c r="L22" t="n">

</xml_diff>